<commit_message>
feat: update dictionary Excel import format
</commit_message>
<xml_diff>
--- a/docs/templates/name_dictionaries_empty.xlsx
+++ b/docs/templates/name_dictionaries_empty.xlsx
@@ -7,9 +7,12 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="surnames" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="names" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="patronymics" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="surname_male" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="names_male" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="patronimic_male" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="surname_female" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="names_female" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="patronimic_female" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -134,47 +137,42 @@
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0">
       <text>
-        <t>Обов'язкове текстове поле. sex: male або female. base_form дорівнює nominative.</t>
+        <t>Обов'язкове текстове поле. Стать і категорія визначені аркушем. base_form дорівнює nominative.</t>
       </text>
     </comment>
     <comment ref="B1" authorId="0" shapeId="0">
       <text>
-        <t>Обов'язкове текстове поле. sex: male або female. base_form дорівнює nominative.</t>
+        <t>Обов'язкове текстове поле. Стать і категорія визначені аркушем. base_form дорівнює nominative.</t>
       </text>
     </comment>
     <comment ref="C1" authorId="0" shapeId="0">
       <text>
-        <t>Обов'язкове текстове поле. sex: male або female. base_form дорівнює nominative.</t>
+        <t>Обов'язкове текстове поле. Стать і категорія визначені аркушем. base_form дорівнює nominative.</t>
       </text>
     </comment>
     <comment ref="D1" authorId="0" shapeId="0">
       <text>
-        <t>Обов'язкове текстове поле. sex: male або female. base_form дорівнює nominative.</t>
+        <t>Обов'язкове текстове поле. Стать і категорія визначені аркушем. base_form дорівнює nominative.</t>
       </text>
     </comment>
     <comment ref="E1" authorId="0" shapeId="0">
       <text>
-        <t>Обов'язкове текстове поле. sex: male або female. base_form дорівнює nominative.</t>
+        <t>Обов'язкове текстове поле. Стать і категорія визначені аркушем. base_form дорівнює nominative.</t>
       </text>
     </comment>
     <comment ref="F1" authorId="0" shapeId="0">
       <text>
-        <t>Обов'язкове текстове поле. sex: male або female. base_form дорівнює nominative.</t>
+        <t>Обов'язкове текстове поле. Стать і категорія визначені аркушем. base_form дорівнює nominative.</t>
       </text>
     </comment>
     <comment ref="G1" authorId="0" shapeId="0">
       <text>
-        <t>Обов'язкове текстове поле. sex: male або female. base_form дорівнює nominative.</t>
+        <t>Обов'язкове текстове поле. Стать і категорія визначені аркушем. base_form дорівнює nominative.</t>
       </text>
     </comment>
     <comment ref="H1" authorId="0" shapeId="0">
       <text>
-        <t>Обов'язкове текстове поле. sex: male або female. base_form дорівнює nominative.</t>
-      </text>
-    </comment>
-    <comment ref="I1" authorId="0" shapeId="0">
-      <text>
-        <t>Обов'язкове текстове поле. sex: male або female. base_form дорівнює nominative.</t>
+        <t>Обов'язкове текстове поле. Стать і категорія визначені аркушем. base_form дорівнює nominative.</t>
       </text>
     </comment>
   </commentList>
@@ -189,47 +187,42 @@
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0">
       <text>
-        <t>Обов'язкове текстове поле. sex: male або female. base_form дорівнює nominative.</t>
+        <t>Обов'язкове текстове поле. Стать і категорія визначені аркушем. base_form дорівнює nominative.</t>
       </text>
     </comment>
     <comment ref="B1" authorId="0" shapeId="0">
       <text>
-        <t>Обов'язкове текстове поле. sex: male або female. base_form дорівнює nominative.</t>
+        <t>Обов'язкове текстове поле. Стать і категорія визначені аркушем. base_form дорівнює nominative.</t>
       </text>
     </comment>
     <comment ref="C1" authorId="0" shapeId="0">
       <text>
-        <t>Обов'язкове текстове поле. sex: male або female. base_form дорівнює nominative.</t>
+        <t>Обов'язкове текстове поле. Стать і категорія визначені аркушем. base_form дорівнює nominative.</t>
       </text>
     </comment>
     <comment ref="D1" authorId="0" shapeId="0">
       <text>
-        <t>Обов'язкове текстове поле. sex: male або female. base_form дорівнює nominative.</t>
+        <t>Обов'язкове текстове поле. Стать і категорія визначені аркушем. base_form дорівнює nominative.</t>
       </text>
     </comment>
     <comment ref="E1" authorId="0" shapeId="0">
       <text>
-        <t>Обов'язкове текстове поле. sex: male або female. base_form дорівнює nominative.</t>
+        <t>Обов'язкове текстове поле. Стать і категорія визначені аркушем. base_form дорівнює nominative.</t>
       </text>
     </comment>
     <comment ref="F1" authorId="0" shapeId="0">
       <text>
-        <t>Обов'язкове текстове поле. sex: male або female. base_form дорівнює nominative.</t>
+        <t>Обов'язкове текстове поле. Стать і категорія визначені аркушем. base_form дорівнює nominative.</t>
       </text>
     </comment>
     <comment ref="G1" authorId="0" shapeId="0">
       <text>
-        <t>Обов'язкове текстове поле. sex: male або female. base_form дорівнює nominative.</t>
+        <t>Обов'язкове текстове поле. Стать і категорія визначені аркушем. base_form дорівнює nominative.</t>
       </text>
     </comment>
     <comment ref="H1" authorId="0" shapeId="0">
       <text>
-        <t>Обов'язкове текстове поле. sex: male або female. base_form дорівнює nominative.</t>
-      </text>
-    </comment>
-    <comment ref="I1" authorId="0" shapeId="0">
-      <text>
-        <t>Обов'язкове текстове поле. sex: male або female. base_form дорівнює nominative.</t>
+        <t>Обов'язкове текстове поле. Стать і категорія визначені аркушем. base_form дорівнює nominative.</t>
       </text>
     </comment>
   </commentList>
@@ -244,47 +237,192 @@
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0">
       <text>
-        <t>Обов'язкове текстове поле. sex: male або female. base_form дорівнює nominative.</t>
+        <t>Обов'язкове текстове поле. Стать і категорія визначені аркушем. base_form дорівнює nominative.</t>
       </text>
     </comment>
     <comment ref="B1" authorId="0" shapeId="0">
       <text>
-        <t>Обов'язкове текстове поле. sex: male або female. base_form дорівнює nominative.</t>
+        <t>Обов'язкове текстове поле. Стать і категорія визначені аркушем. base_form дорівнює nominative.</t>
       </text>
     </comment>
     <comment ref="C1" authorId="0" shapeId="0">
       <text>
-        <t>Обов'язкове текстове поле. sex: male або female. base_form дорівнює nominative.</t>
+        <t>Обов'язкове текстове поле. Стать і категорія визначені аркушем. base_form дорівнює nominative.</t>
       </text>
     </comment>
     <comment ref="D1" authorId="0" shapeId="0">
       <text>
-        <t>Обов'язкове текстове поле. sex: male або female. base_form дорівнює nominative.</t>
+        <t>Обов'язкове текстове поле. Стать і категорія визначені аркушем. base_form дорівнює nominative.</t>
       </text>
     </comment>
     <comment ref="E1" authorId="0" shapeId="0">
       <text>
-        <t>Обов'язкове текстове поле. sex: male або female. base_form дорівнює nominative.</t>
+        <t>Обов'язкове текстове поле. Стать і категорія визначені аркушем. base_form дорівнює nominative.</t>
       </text>
     </comment>
     <comment ref="F1" authorId="0" shapeId="0">
       <text>
-        <t>Обов'язкове текстове поле. sex: male або female. base_form дорівнює nominative.</t>
+        <t>Обов'язкове текстове поле. Стать і категорія визначені аркушем. base_form дорівнює nominative.</t>
       </text>
     </comment>
     <comment ref="G1" authorId="0" shapeId="0">
       <text>
-        <t>Обов'язкове текстове поле. sex: male або female. base_form дорівнює nominative.</t>
+        <t>Обов'язкове текстове поле. Стать і категорія визначені аркушем. base_form дорівнює nominative.</t>
       </text>
     </comment>
     <comment ref="H1" authorId="0" shapeId="0">
       <text>
-        <t>Обов'язкове текстове поле. sex: male або female. base_form дорівнює nominative.</t>
-      </text>
-    </comment>
-    <comment ref="I1" authorId="0" shapeId="0">
-      <text>
-        <t>Обов'язкове текстове поле. sex: male або female. base_form дорівнює nominative.</t>
+        <t>Обов'язкове текстове поле. Стать і категорія визначені аркушем. base_form дорівнює nominative.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment4.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>project_2</author>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0" shapeId="0">
+      <text>
+        <t>Обов'язкове текстове поле. Стать і категорія визначені аркушем. base_form дорівнює nominative.</t>
+      </text>
+    </comment>
+    <comment ref="B1" authorId="0" shapeId="0">
+      <text>
+        <t>Обов'язкове текстове поле. Стать і категорія визначені аркушем. base_form дорівнює nominative.</t>
+      </text>
+    </comment>
+    <comment ref="C1" authorId="0" shapeId="0">
+      <text>
+        <t>Обов'язкове текстове поле. Стать і категорія визначені аркушем. base_form дорівнює nominative.</t>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0" shapeId="0">
+      <text>
+        <t>Обов'язкове текстове поле. Стать і категорія визначені аркушем. base_form дорівнює nominative.</t>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="0" shapeId="0">
+      <text>
+        <t>Обов'язкове текстове поле. Стать і категорія визначені аркушем. base_form дорівнює nominative.</t>
+      </text>
+    </comment>
+    <comment ref="F1" authorId="0" shapeId="0">
+      <text>
+        <t>Обов'язкове текстове поле. Стать і категорія визначені аркушем. base_form дорівнює nominative.</t>
+      </text>
+    </comment>
+    <comment ref="G1" authorId="0" shapeId="0">
+      <text>
+        <t>Обов'язкове текстове поле. Стать і категорія визначені аркушем. base_form дорівнює nominative.</t>
+      </text>
+    </comment>
+    <comment ref="H1" authorId="0" shapeId="0">
+      <text>
+        <t>Обов'язкове текстове поле. Стать і категорія визначені аркушем. base_form дорівнює nominative.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment5.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>project_2</author>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0" shapeId="0">
+      <text>
+        <t>Обов'язкове текстове поле. Стать і категорія визначені аркушем. base_form дорівнює nominative.</t>
+      </text>
+    </comment>
+    <comment ref="B1" authorId="0" shapeId="0">
+      <text>
+        <t>Обов'язкове текстове поле. Стать і категорія визначені аркушем. base_form дорівнює nominative.</t>
+      </text>
+    </comment>
+    <comment ref="C1" authorId="0" shapeId="0">
+      <text>
+        <t>Обов'язкове текстове поле. Стать і категорія визначені аркушем. base_form дорівнює nominative.</t>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0" shapeId="0">
+      <text>
+        <t>Обов'язкове текстове поле. Стать і категорія визначені аркушем. base_form дорівнює nominative.</t>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="0" shapeId="0">
+      <text>
+        <t>Обов'язкове текстове поле. Стать і категорія визначені аркушем. base_form дорівнює nominative.</t>
+      </text>
+    </comment>
+    <comment ref="F1" authorId="0" shapeId="0">
+      <text>
+        <t>Обов'язкове текстове поле. Стать і категорія визначені аркушем. base_form дорівнює nominative.</t>
+      </text>
+    </comment>
+    <comment ref="G1" authorId="0" shapeId="0">
+      <text>
+        <t>Обов'язкове текстове поле. Стать і категорія визначені аркушем. base_form дорівнює nominative.</t>
+      </text>
+    </comment>
+    <comment ref="H1" authorId="0" shapeId="0">
+      <text>
+        <t>Обов'язкове текстове поле. Стать і категорія визначені аркушем. base_form дорівнює nominative.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment6.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>project_2</author>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0" shapeId="0">
+      <text>
+        <t>Обов'язкове текстове поле. Стать і категорія визначені аркушем. base_form дорівнює nominative.</t>
+      </text>
+    </comment>
+    <comment ref="B1" authorId="0" shapeId="0">
+      <text>
+        <t>Обов'язкове текстове поле. Стать і категорія визначені аркушем. base_form дорівнює nominative.</t>
+      </text>
+    </comment>
+    <comment ref="C1" authorId="0" shapeId="0">
+      <text>
+        <t>Обов'язкове текстове поле. Стать і категорія визначені аркушем. base_form дорівнює nominative.</t>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0" shapeId="0">
+      <text>
+        <t>Обов'язкове текстове поле. Стать і категорія визначені аркушем. base_form дорівнює nominative.</t>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="0" shapeId="0">
+      <text>
+        <t>Обов'язкове текстове поле. Стать і категорія визначені аркушем. base_form дорівнює nominative.</t>
+      </text>
+    </comment>
+    <comment ref="F1" authorId="0" shapeId="0">
+      <text>
+        <t>Обов'язкове текстове поле. Стать і категорія визначені аркушем. base_form дорівнює nominative.</t>
+      </text>
+    </comment>
+    <comment ref="G1" authorId="0" shapeId="0">
+      <text>
+        <t>Обов'язкове текстове поле. Стать і категорія визначені аркушем. base_form дорівнює nominative.</t>
+      </text>
+    </comment>
+    <comment ref="H1" authorId="0" shapeId="0">
+      <text>
+        <t>Обов'язкове текстове поле. Стать і категорія визначені аркушем. base_form дорівнює nominative.</t>
       </text>
     </comment>
   </commentList>
@@ -580,7 +718,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -591,7 +729,6 @@
     <col width="24" customWidth="1" min="6" max="6"/>
     <col width="24" customWidth="1" min="7" max="7"/>
     <col width="24" customWidth="1" min="8" max="8"/>
-    <col width="24" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -602,51 +739,83 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>sex</t>
+          <t>nominative</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>nominative</t>
+          <t>genitive</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>genitive</t>
+          <t>dative</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>dative</t>
+          <t>accusative</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>accusative</t>
+          <t>instrumental</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>instrumental</t>
+          <t>locative</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>locative</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
           <t>vocative</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Основна форма</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Називний</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Родовий</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Давальний</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Знахідний</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Орудний</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Місцевий</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Кличний</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="1">
-    <dataValidation sqref="B2:B10001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Стать не визначається автоматично" error="Вкажіть male або female." type="list">
-      <formula1>"male,female"</formula1>
-    </dataValidation>
-  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
@@ -658,7 +827,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -669,7 +838,6 @@
     <col width="24" customWidth="1" min="6" max="6"/>
     <col width="24" customWidth="1" min="7" max="7"/>
     <col width="24" customWidth="1" min="8" max="8"/>
-    <col width="24" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -680,51 +848,83 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>sex</t>
+          <t>nominative</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>nominative</t>
+          <t>genitive</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>genitive</t>
+          <t>dative</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>dative</t>
+          <t>accusative</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>accusative</t>
+          <t>instrumental</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>instrumental</t>
+          <t>locative</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>locative</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
           <t>vocative</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Основна форма</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Називний</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Родовий</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Давальний</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Знахідний</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Орудний</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Місцевий</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Кличний</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="1">
-    <dataValidation sqref="B2:B10001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Стать не визначається автоматично" error="Вкажіть male або female." type="list">
-      <formula1>"male,female"</formula1>
-    </dataValidation>
-  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
@@ -736,7 +936,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -747,7 +947,6 @@
     <col width="24" customWidth="1" min="6" max="6"/>
     <col width="24" customWidth="1" min="7" max="7"/>
     <col width="24" customWidth="1" min="8" max="8"/>
-    <col width="24" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -758,51 +957,410 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>sex</t>
+          <t>nominative</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>nominative</t>
+          <t>genitive</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>genitive</t>
+          <t>dative</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>dative</t>
+          <t>accusative</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>accusative</t>
+          <t>instrumental</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>instrumental</t>
+          <t>locative</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>locative</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
           <t>vocative</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Основна форма</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Називний</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Родовий</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Давальний</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Знахідний</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Орудний</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Місцевий</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Кличний</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="1">
-    <dataValidation sqref="B2:B10001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Стать не визначається автоматично" error="Вкажіть male або female." type="list">
-      <formula1>"male,female"</formula1>
-    </dataValidation>
-  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>base_form</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>nominative</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>genitive</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>dative</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>accusative</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>instrumental</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>locative</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>vocative</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Основна форма</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Називний</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Родовий</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Давальний</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Знахідний</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Орудний</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Місцевий</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Кличний</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>base_form</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>nominative</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>genitive</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>dative</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>accusative</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>instrumental</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>locative</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>vocative</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Основна форма</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Називний</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Родовий</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Давальний</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Знахідний</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Орудний</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Місцевий</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Кличний</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>base_form</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>nominative</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>genitive</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>dative</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>accusative</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>instrumental</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>locative</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>vocative</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Основна форма</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Називний</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Родовий</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Давальний</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Знахідний</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Орудний</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Місцевий</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Кличний</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>

</xml_diff>